<commit_message>
Cosmetici: autorrevisão de 09/2026 e cruzamentos automáticos
- CT-e: crédito do frete segue a natureza da NF-e transportada (CT-e 5597996
  do pincel/uso e consumo deixa de creditar R$ 36,18; ICMS 09/2026 9.996,19)
- revisao.py: industrialização x retorno (insumo em 5124/6124 em duplicidade
  com 5902/6902, 5124 sem insumo do cliente, retorno citando NF errada),
  contribuinte com IE como consumidor final, CNPJ com UF diferente, CFOP de
  revenda com IPI, diferimento 5124, grupo IPI, remessas sem retorno e
  retenções das NFS-e tomadas (--nfse RelatorioNFS_ABRASF)
- aba Checklist na planilha de apuração; checklist de 09/2026
- testes sintéticos para os novos cruzamentos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GpFQAF7UfcTJUBPm398Z8s
</commit_message>
<xml_diff>
--- a/Cosmetici/Fiscal/2026-09/Creditos_Entradas_Cosmetici_09-2026.xlsx
+++ b/Cosmetici/Fiscal/2026-09/Creditos_Entradas_Cosmetici_09-2026.xlsx
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>185.32</v>
+        <v>149.14</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>6357.94</v>
+        <v>6321.76</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
@@ -11201,7 +11201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11213,6 +11213,7 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11268,41 +11269,51 @@
           <t>Observação</t>
         </is>
       </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>NF-e transportada</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="7" t="n">
         <v>5597996</v>
       </c>
-      <c r="B4" s="15" t="n">
+      <c r="B4" s="18" t="n">
         <v>46269</v>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>CAXIAS DO SUL - EXPRESSO SAO MIGUEL S/A</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>2352</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="8" t="n">
         <v>301.49</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="8" t="n">
         <v>36.18</v>
       </c>
-      <c r="G4" s="6" t="n">
-        <v>36.18</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>XML</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Frete de compra/venda tomado pela COSMETICI</t>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Frete de compra de outras: sem crédito - o crédito do frete segue a mercadoria (uso e consumo/outras não creditam - LC 87/96 art. 33, I). ICMS R$ 36.18 não aproveitado</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>NF 2564 (outras)</t>
         </is>
       </c>
     </row>
@@ -11339,7 +11350,12 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Frete de compra/venda tomado pela COSMETICI</t>
+          <t>Frete de compra de insumo</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>NF 30338 (insumo)</t>
         </is>
       </c>
     </row>
@@ -11376,7 +11392,12 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Frete de compra/venda tomado pela COSMETICI</t>
+          <t>Frete de compra de insumo</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>NF 117690 (insumo)</t>
         </is>
       </c>
     </row>
@@ -11413,7 +11434,12 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Frete de compra/venda tomado pela COSMETICI</t>
+          <t>Frete de compra de insumo</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>NF 141811 (insumo)</t>
         </is>
       </c>
     </row>
@@ -11450,7 +11476,12 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Frete de compra/venda tomado pela COSMETICI</t>
+          <t>Frete de compra de insumo</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>NF 19303 (insumo)</t>
         </is>
       </c>
     </row>
@@ -11490,6 +11521,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -11527,6 +11559,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -11564,6 +11597,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -11601,6 +11635,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -11638,6 +11673,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -11675,6 +11711,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -11712,6 +11749,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -11749,6 +11787,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -11786,6 +11825,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -11823,6 +11863,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -11860,6 +11901,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -11897,6 +11939,7 @@
           <t>Frete de venda (Cosmetici tomadora) - XML não está na pasta</t>
         </is>
       </c>
+      <c r="J20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -11934,6 +11977,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -11971,6 +12015,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -12008,6 +12053,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -12045,6 +12091,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -12082,6 +12129,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -12119,6 +12167,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -12156,6 +12205,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -12193,6 +12243,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -12230,6 +12281,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -12267,6 +12319,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -12304,6 +12357,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -12341,6 +12395,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -12378,6 +12433,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -12415,6 +12471,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -12452,6 +12509,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -12489,6 +12547,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -12526,6 +12585,7 @@
           <t>Envio de pedido da GULA COSMETICOS a consumidor final com a Cosmetici no CT-e - frete de operação de terceiro: NÃO creditar sem confirmar</t>
         </is>
       </c>
+      <c r="J37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
@@ -12550,6 +12610,7 @@
       </c>
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="9" t="inlineStr"/>
+      <c r="J38" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>